<commit_message>
Answer sheets: in-sheet instructions, plain headers, tooltip prompts; scorer reads xlsx natively (end-to-end tested incl. float verse cells)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agent/data/eval/packets/Response_Sheet_1.xlsx
+++ b/agent/data/eval/packets/Response_Sheet_1.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <i val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -54,9 +57,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
@@ -425,316 +433,326 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="58" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="44" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>verse</t>
+          <t>For each verse (see the PDF packet), answer the three questions by choosing A, B, C, or tie in each column. Leave blank only if no option is acceptable, and please say why in Comments.</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>term_fidelity</t>
+          <t>Verse</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>compound_resolution</t>
+          <t>Q1: Technical terms (A/B/C/tie)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>overall</t>
+          <t>Q2: Compounds (A/B/C/tie)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>comments</t>
+          <t>Q3: Overall (A/B/C/tie)</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Comments (optional)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr"/>
-      <c r="E21" s="2" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
-      <c r="E23" s="2" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
-      <c r="E25" s="2" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" s="2" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" s="2" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" s="2" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B2:D31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B3:D32" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Please enter A, B, C, or tie" promptTitle="Your judgment" prompt="Choose A, B, C, or tie" type="list">
       <formula1>"A,B,C,tie"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>